<commit_message>
Update estimation checklist alignment
</commit_message>
<xml_diff>
--- a/downloads/estimation-checksheet.xlsx
+++ b/downloads/estimation-checksheet.xlsx
@@ -138,7 +138,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ユーザ数: _____　端末数: _____　拠点数: _____　対象機器数: _____</t>
+          <t>ユーザ数: _____　端末数: _____　拠点数: _____　VPN装置数: _____　AP台数: _____　SSID数: _____　VLAN数: _____</t>
         </is>
       </c>
     </row>
@@ -203,12 +203,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VPN方式: __________　認証方式: __________　既存ポリシー: □ あり　□ なし</t>
+          <t>VPN方式: __________　認証方式: __________　VPNクライアント: __________　ライセンス: □ 確認済　□ 要確認　既存ポリシー: □ あり　□ なし</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>利用中のVPNクライアント、ユーザ / グループ制御の有無を記入する</t>
+          <t>利用中のVPNクライアント、ライセンス要件、ユーザ / グループ制御の有無を記入する</t>
         </is>
       </c>
     </row>
@@ -220,7 +220,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SSID数: _____　VLAN: □ あり　□ なし　AP / コントローラ: __________</t>
+          <t>SSID数: _____　VLAN数: _____　AP台数: _____　AP / コントローラ: __________</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -232,84 +232,101 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ネットワーク</t>
+          <t>作業条件</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>固定IP / DDNS: __________　NAT: □ あり　□ なし　FW / ACL変更: □ 必要　□ 不要</t>
+          <t>リモート作業: □ 可　□ 不可　変更申請: □ 要　□ 不要　立ち会い: □ 要　□ 不要</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>RADIUS通信経路、DNS / DDNS、経路上の制御を記入する</t>
+          <t>作業場所、申請フロー、立ち会い体制を記入する</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>機器設定ファイル</t>
+          <t>ネットワーク</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>提供可否: □ 可能　□ 不可　□ 要調整　対象機器: __________　マスキング: □ 済　□ 未</t>
+          <t>固定IP / DDNS: __________　NAT: □ あり　□ なし　FW / ACL変更: □ 必要　□ 不要</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>既存VPN、インターフェース、アドレスプール、ポリシー、証明書、RADIUS設定を読み取れる範囲で提供してもらう</t>
+          <t>RADIUS通信経路、DNS / DDNS、経路上の制御を記入する</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ID管理</t>
+          <t>機器設定ファイル</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>□ Active Directory　□ Microsoft Entra ID　□ その他IdP　□ ID管理なし</t>
+          <t>提供可否: □ 可能　□ 不可　□ 要調整　対象機器: __________　マスキング: □ 済　□ 未</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ユーザ登録方式やSCIM要否に影響する前提を記入する</t>
+          <t>既存VPN、インターフェース、アドレスプール、ポリシー、証明書、RADIUS設定を読み取れる範囲で提供してもらう</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>証明書</t>
+          <t>ID管理</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>既存CA: □ あり　□ なし　端末証明書: □ あり　□ なし　Intune: □ あり　□ なし</t>
+          <t>□ Active Directory　□ Microsoft Entra ID　□ その他IdP　□ ID管理なし</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>証明書配布方法、既存証明書の継続利用可否を記入する</t>
+          <t>ユーザ登録方式やSCIM要否に影響する前提を記入する</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>証明書</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>既存CA: □ あり　□ なし　端末証明書: □ あり　□ なし　Intune: □ あり　□ なし</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>証明書配布方法、既存証明書の継続利用可否を記入する</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>端末展開</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>対象OS: □ Windows　□ macOS　□ iOS / iPadOS　□ Android　□ その他
 端末管理: □ MDM　□ 管理者　□ 利用者　□ 不明</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>VPNクライアント、無線プロファイル、証明書の展開方法を記入する</t>
         </is>
@@ -581,7 +598,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>機器のファームウェア、設定ガイド適合、RADIUS属性の確定</t>
+          <t>機器のファームウェア、ライセンス、設定ガイド適合、RADIUS属性、VPNクライアント要件の確定</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -625,7 +642,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>作業時間帯、切り戻し条件、受け入れ条件、運用 / サポート範囲の確定</t>
+          <t>リモート作業可否、変更申請、立ち会い要否、作業時間帯、切り戻し条件、受け入れ条件、運用 / サポート範囲の確定</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>

<commit_message>
Publish latest training docs
</commit_message>
<xml_diff>
--- a/downloads/estimation-checksheet.xlsx
+++ b/downloads/estimation-checksheet.xlsx
@@ -162,7 +162,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>利用開始希望日: _____　作業可能時間帯: _____　PoC: □ 不要　□ 必要（理由: _____）</t>
+          <t>利用開始希望日: _____　作業可能時間帯: _____　PoC: □ 不要　□ 要（理由: _____）</t>
         </is>
       </c>
     </row>
@@ -203,7 +203,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VPN方式: __________　認証方式: __________　VPNクライアント: __________　ライセンス: □ 確認済　□ 要確認　既存ポリシー: □ あり　□ なし</t>
+          <t>VPN方式: __________　認証方式: __________　VPNクライアント: __________　ライセンス: □ 確認済　□ 要確認　既存ポリシー: □ 有　□ 無</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -254,7 +254,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>固定IP / DDNS: __________　NAT: □ あり　□ なし　FW / ACL変更: □ 必要　□ 不要</t>
+          <t>固定IP / DDNS: __________　NAT: □ 有　□ 無　FW / ACL変更: □ 要　□ 不要</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -305,7 +305,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>既存CA: □ あり　□ なし　端末証明書: □ あり　□ なし　Intune: □ あり　□ なし</t>
+          <t>既存CA: □ 有　□ 無　端末証明書: □ 有　□ 無　Intune: □ 有　□ 無</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">

</xml_diff>